<commit_message>
correção do check, funcionando o cadastro de clientes
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="162">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -283,6 +283,9 @@
   </si>
   <si>
     <t xml:space="preserve">Campo de status do marca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK (1,2)</t>
   </si>
   <si>
     <t xml:space="preserve">modelo</t>
@@ -1875,7 +1878,7 @@
         <v>23</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="H43" s="11" t="s">
         <v>48</v>
@@ -1886,7 +1889,7 @@
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>20</v>
@@ -1906,15 +1909,15 @@
       </c>
       <c r="H44" s="11"/>
       <c r="I44" s="10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>27</v>
@@ -1927,12 +1930,12 @@
       <c r="G45" s="8"/>
       <c r="H45" s="7"/>
       <c r="I45" s="10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>32</v>
@@ -1950,12 +1953,12 @@
       </c>
       <c r="H46" s="7"/>
       <c r="I46" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>44</v>
@@ -1980,7 +1983,7 @@
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>46</v>
@@ -2007,7 +2010,7 @@
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B49" s="15" t="s">
         <v>20</v>
@@ -2027,15 +2030,15 @@
       </c>
       <c r="H49" s="11"/>
       <c r="I49" s="10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>27</v>
@@ -2048,12 +2051,12 @@
       <c r="G50" s="8"/>
       <c r="H50" s="7"/>
       <c r="I50" s="10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B51" s="11" t="s">
         <v>32</v>
@@ -2071,12 +2074,12 @@
       </c>
       <c r="H51" s="7"/>
       <c r="I51" s="10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B52" s="11" t="s">
         <v>44</v>
@@ -2101,7 +2104,7 @@
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B53" s="11" t="s">
         <v>46</v>
@@ -2391,89 +2394,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2481,7 +2484,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>12</v>
@@ -2496,10 +2499,10 @@
         <v>15</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>18</v>
@@ -2507,16 +2510,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>22</v>
@@ -2525,131 +2528,131 @@
         <v>23</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>23</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>23</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>23</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>68</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>35</v>
@@ -2658,27 +2661,27 @@
         <v>23</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>22</v>
@@ -2687,65 +2690,65 @@
         <v>23</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>23</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>23</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>
@@ -2780,7 +2783,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>35</v>
@@ -2791,23 +2794,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2817,27 +2820,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
inicio tabela ordem de servico
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="162">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -997,7 +997,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -1608,118 +1608,124 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="B32" s="15" t="s">
-        <v>20</v>
+      <c r="A32" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>44</v>
       </c>
       <c r="C32" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D32" s="13"/>
       <c r="E32" s="13" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="F32" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G32" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H32" s="11"/>
-      <c r="I32" s="10" t="s">
-        <v>72</v>
+      <c r="G32" s="12"/>
+      <c r="H32" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
+      <c r="A33" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="F33" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G33" s="8"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="10" t="s">
-        <v>74</v>
+      <c r="G33" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="B34" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
+      <c r="B34" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="F34" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G34" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H34" s="7"/>
+      <c r="G34" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H34" s="11"/>
       <c r="I34" s="10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D35" s="13"/>
-      <c r="E35" s="13" t="s">
-        <v>22</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
       <c r="F35" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G35" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H35" s="11"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="7"/>
       <c r="I35" s="10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>78</v>
+        <v>71</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>32</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D36" s="9"/>
       <c r="E36" s="9"/>
       <c r="F36" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G36" s="8"/>
+      <c r="G36" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="H36" s="7"/>
       <c r="I36" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1727,429 +1733,453 @@
         <v>76</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C37" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+      <c r="E37" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="F37" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G37" s="12"/>
+      <c r="G37" s="12" t="s">
+        <v>24</v>
+      </c>
       <c r="H37" s="11"/>
       <c r="I37" s="10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="s">
+      <c r="A38" s="11" t="s">
         <v>76</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
-      <c r="F38" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>30</v>
-      </c>
+      <c r="F38" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G38" s="8"/>
       <c r="H38" s="7"/>
-      <c r="I38" s="14" t="s">
-        <v>81</v>
+      <c r="I38" s="10" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B39" s="15" t="s">
-        <v>20</v>
+        <v>76</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>32</v>
       </c>
       <c r="C39" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D39" s="13"/>
-      <c r="E39" s="13" t="s">
-        <v>22</v>
-      </c>
+      <c r="E39" s="13"/>
       <c r="F39" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G39" s="12" t="s">
-        <v>24</v>
-      </c>
+      <c r="G39" s="12"/>
       <c r="H39" s="11"/>
       <c r="I39" s="10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
-        <v>82</v>
+      <c r="A40" s="7" t="s">
+        <v>76</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D40" s="9"/>
       <c r="E40" s="9"/>
-      <c r="F40" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G40" s="8"/>
+      <c r="F40" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G40" s="12" t="s">
+        <v>30</v>
+      </c>
       <c r="H40" s="7"/>
-      <c r="I40" s="10" t="s">
-        <v>85</v>
+      <c r="I40" s="14" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B41" s="11" t="s">
+      <c r="B41" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F41" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H41" s="11"/>
+      <c r="I41" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G42" s="8"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B43" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D41" s="9"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G41" s="8" t="n">
+      <c r="C43" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G43" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H41" s="7"/>
-      <c r="I41" s="10" t="s">
+      <c r="H43" s="7"/>
+      <c r="I43" s="10" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
+    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B44" s="11" t="s">
         <v>44</v>
-      </c>
-      <c r="C42" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D42" s="13"/>
-      <c r="E42" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F42" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G42" s="12"/>
-      <c r="H42" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="I42" s="14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C43" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F43" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G43" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="H43" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I43" s="14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B44" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="C44" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D44" s="13"/>
       <c r="E44" s="13" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="F44" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G44" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H44" s="11"/>
-      <c r="I44" s="10" t="s">
-        <v>89</v>
+      <c r="G44" s="12"/>
+      <c r="H44" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I44" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
+      <c r="A45" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="F45" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G45" s="8"/>
-      <c r="H45" s="7"/>
-      <c r="I45" s="10" t="s">
-        <v>91</v>
+      <c r="G45" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H45" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="I45" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F46" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G46" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H46" s="11"/>
+      <c r="I46" s="10" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G47" s="8"/>
+      <c r="H47" s="7"/>
+      <c r="I47" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B48" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C46" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G46" s="8" t="n">
+      <c r="C48" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G48" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H46" s="7"/>
-      <c r="I46" s="10" t="s">
+      <c r="H48" s="7"/>
+      <c r="I48" s="10" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="s">
+    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B49" s="11" t="s">
         <v>44</v>
-      </c>
-      <c r="C47" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D47" s="13"/>
-      <c r="E47" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F47" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G47" s="12"/>
-      <c r="H47" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="I47" s="14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="B48" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="C48" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F48" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G48" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="H48" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="I48" s="14" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="C49" s="12" t="s">
         <v>21</v>
       </c>
       <c r="D49" s="13"/>
       <c r="E49" s="13" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="F49" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G49" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="H49" s="11"/>
-      <c r="I49" s="10" t="s">
-        <v>94</v>
+      <c r="G49" s="12"/>
+      <c r="H49" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I49" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="B50" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="C50" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D50" s="9"/>
-      <c r="E50" s="9"/>
+      <c r="A50" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="13"/>
+      <c r="E50" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="F50" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G50" s="8"/>
-      <c r="H50" s="7"/>
-      <c r="I50" s="10" t="s">
-        <v>96</v>
+      <c r="G50" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H50" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="I50" s="14" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B51" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D51" s="13"/>
+      <c r="E51" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G51" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H51" s="11"/>
+      <c r="I51" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G52" s="8"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B53" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C51" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G51" s="8" t="n">
+      <c r="C53" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G53" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H51" s="7"/>
-      <c r="I51" s="10" t="s">
+      <c r="H53" s="7"/>
+      <c r="I53" s="10" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="7" t="s">
+    <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B52" s="11" t="s">
+      <c r="B54" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C52" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13" t="s">
+      <c r="C54" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D54" s="13"/>
+      <c r="E54" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="F52" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G52" s="12"/>
-      <c r="H52" s="11" t="s">
+      <c r="F54" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G54" s="12"/>
+      <c r="H54" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="I52" s="14" t="s">
+      <c r="I54" s="14" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
+    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="B53" s="11" t="s">
+      <c r="B55" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C53" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13" t="s">
+      <c r="C55" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="F53" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="G53" s="12" t="s">
+      <c r="F55" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="G55" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="H53" s="11" t="s">
+      <c r="H55" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="I53" s="14" t="s">
+      <c r="I55" s="14" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="7"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="9"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="7"/>
-      <c r="I54" s="10"/>
-    </row>
-    <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="11"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="11"/>
-      <c r="I55" s="14"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7"/>
@@ -2349,17 +2379,39 @@
       <c r="H73" s="11"/>
       <c r="I73" s="14"/>
     </row>
+    <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="7"/>
+      <c r="B74" s="7"/>
+      <c r="C74" s="8"/>
+      <c r="D74" s="9"/>
+      <c r="E74" s="9"/>
+      <c r="F74" s="9"/>
+      <c r="G74" s="8"/>
+      <c r="H74" s="7"/>
+      <c r="I74" s="10"/>
+    </row>
+    <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="11"/>
+      <c r="B75" s="11"/>
+      <c r="C75" s="12"/>
+      <c r="D75" s="13"/>
+      <c r="E75" s="13"/>
+      <c r="F75" s="13"/>
+      <c r="G75" s="12"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="14"/>
+    </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C73" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C75" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E73" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E75" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F73" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F75" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>